<commit_message>
Late update of work_reference.xlsx
</commit_message>
<xml_diff>
--- a/work_reference.xlsx
+++ b/work_reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Oskari\AppData\Roaming\Autodesk\Autodesk Fusion 360\API\AddIns\BodyCount\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9329FBD0-56B6-42C2-A046-ADB0572494E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D498CDB7-4057-4696-BB2C-B59828E63EE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7215" yWindow="3795" windowWidth="33450" windowHeight="17085" xr2:uid="{C175BA65-C788-4E3B-AACC-D273C035F0F3}"/>
+    <workbookView xWindow="10665" yWindow="2115" windowWidth="33450" windowHeight="17085" xr2:uid="{C175BA65-C788-4E3B-AACC-D273C035F0F3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -419,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00CAE36-1E69-4377-8A1B-200D917D115F}">
-  <dimension ref="B1:I20"/>
+  <dimension ref="B1:I21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -459,7 +459,7 @@
       </c>
       <c r="C3" s="4">
         <f>SUM(I:I)</f>
-        <v>1.5173611111111114</v>
+        <v>1.5381944444444446</v>
       </c>
       <c r="F3" s="5">
         <v>45602</v>
@@ -481,7 +481,7 @@
       </c>
       <c r="C4" s="2">
         <f>C3*24*C2</f>
-        <v>9104.1666666666679</v>
+        <v>9229.1666666666679</v>
       </c>
       <c r="F4" s="5"/>
       <c r="G4" s="1">
@@ -491,7 +491,7 @@
         <v>0.94444444444444442</v>
       </c>
       <c r="I4" s="1">
-        <f t="shared" ref="I4:I20" si="0">H4-G4</f>
+        <f t="shared" ref="I4:I21" si="0">H4-G4</f>
         <v>9.027777777777779E-2</v>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="C5" s="2">
         <f>C4*0.68</f>
-        <v>6190.8333333333348</v>
+        <v>6275.8333333333348</v>
       </c>
       <c r="F5" s="5">
         <v>45605</v>
@@ -736,6 +736,21 @@
       <c r="I20" s="1">
         <f t="shared" si="0"/>
         <v>2.0833333333333259E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F21" s="3">
+        <v>45743</v>
+      </c>
+      <c r="G21" s="1">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="H21" s="1">
+        <v>0.875</v>
+      </c>
+      <c r="I21" s="1">
+        <f t="shared" si="0"/>
+        <v>2.083333333333337E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>